<commit_message>
app modificado por 4ta vez
</commit_message>
<xml_diff>
--- a/resultados.xlsx
+++ b/resultados.xlsx
@@ -463,7 +463,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>No se encontró el input del DNI después de 15 segundos</t>
+          <t>No se encontró ningún input en la página</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -485,7 +485,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>No se encontró el input del DNI después de 15 segundos</t>
+          <t>No se encontró ningún input en la página</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -507,7 +507,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>No se encontró el input del DNI después de 15 segundos</t>
+          <t>No se encontró ningún input en la página</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">

</xml_diff>

<commit_message>
errores solucionados y codigo funcionando
</commit_message>
<xml_diff>
--- a/resultados.xlsx
+++ b/resultados.xlsx
@@ -458,17 +458,17 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>ERROR</t>
+          <t>SI</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>No se encontró ningún input en la página</t>
+          <t>No encontrada</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>No encontrada</t>
         </is>
       </c>
     </row>
@@ -480,17 +480,17 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>ERROR</t>
+          <t>SI</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>No se encontró ningún input en la página</t>
+          <t>No encontrada</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>No encontrada</t>
         </is>
       </c>
     </row>
@@ -502,17 +502,17 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>ERROR</t>
+          <t>SI</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>No se encontró ningún input en la página</t>
+          <t>No encontrada</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>No encontrada</t>
         </is>
       </c>
     </row>

</xml_diff>